<commit_message>
Update product catalog prices, add delivery messaging on Home and About sections
</commit_message>
<xml_diff>
--- a/GREEN CARE (2).xlsx
+++ b/GREEN CARE (2).xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caana\Music\greencare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9C90CC-22F2-45D2-9E8E-937D981A9D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C561BD09-5E7A-4EEC-973C-D133C32CA56A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8C521C81-544A-422E-B8E9-ACD18C8FF525}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5556" xr2:uid="{8C521C81-544A-422E-B8E9-ACD18C8FF525}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="122">
   <si>
     <t>NO</t>
   </si>
@@ -78,9 +78,6 @@
     <t>DUSTBIN COVER</t>
   </si>
   <si>
-    <t>LATEX GLOVES</t>
-  </si>
-  <si>
     <t>NITRAL GLOVES</t>
   </si>
   <si>
@@ -117,48 +114,21 @@
     <t>BROWN TAPE</t>
   </si>
   <si>
-    <t>PAPER ROLL</t>
-  </si>
-  <si>
     <t>SCOTCH BRITE</t>
   </si>
   <si>
     <t>STEEL WOOL</t>
   </si>
   <si>
-    <t>WOODEN SPOON 110 MM</t>
-  </si>
-  <si>
     <t>WOODEN SPOON 160 MM</t>
   </si>
   <si>
-    <t>WOODEN STIRER 160 MM</t>
-  </si>
-  <si>
     <t>WOODEN FORK 160 MM</t>
   </si>
   <si>
-    <t>WOODEN FORK 110 MM</t>
-  </si>
-  <si>
-    <t>PAPER CUP 150 ML</t>
-  </si>
-  <si>
-    <t>PAPER CUP 210 ML</t>
-  </si>
-  <si>
-    <t>PAPER CUP 250 ML</t>
-  </si>
-  <si>
-    <t>PAPER CUP 350 ML</t>
-  </si>
-  <si>
     <t>DISH WASH 5 LTR</t>
   </si>
   <si>
-    <t>FOAM SOAP 5 LTR</t>
-  </si>
-  <si>
     <t>HAND WASH 5 LTR</t>
   </si>
   <si>
@@ -186,12 +156,6 @@
     <t>M FOLD NAPKIN</t>
   </si>
   <si>
-    <t>MOPE</t>
-  </si>
-  <si>
-    <t>WIPER</t>
-  </si>
-  <si>
     <t>SCRUBBING BRUSH</t>
   </si>
   <si>
@@ -213,15 +177,9 @@
     <t>LOBBY DUST PAN</t>
   </si>
   <si>
-    <t>BUCKET</t>
-  </si>
-  <si>
     <t>BROOMS</t>
   </si>
   <si>
-    <t>TABLE CLEANING SPONGE</t>
-  </si>
-  <si>
     <t>DUSTBIN</t>
   </si>
   <si>
@@ -255,9 +213,6 @@
     <t>GST NO  32APYPJ7697H1Z1</t>
   </si>
   <si>
-    <t>PAPER PLATE SMALL</t>
-  </si>
-  <si>
     <t>PAPER PLATE BIG</t>
   </si>
   <si>
@@ -288,9 +243,6 @@
     <t>ALUMINIUM CONTAINER 250 ML</t>
   </si>
   <si>
-    <t xml:space="preserve">SILVER COVER </t>
-  </si>
-  <si>
     <t>GEL FUEL 200 gm</t>
   </si>
   <si>
@@ -306,15 +258,6 @@
     <t>PLASTIC CONTAINER 250 ML</t>
   </si>
   <si>
-    <t>PLASTIC CONTAINER 400 ML</t>
-  </si>
-  <si>
-    <t>PLASTIC CONTAINER 500 ML</t>
-  </si>
-  <si>
-    <t>PLASTIC CONTAINER 1000 ML</t>
-  </si>
-  <si>
     <t>PLASTIC CONTAINER 500  ML SQURE</t>
   </si>
   <si>
@@ -324,15 +267,9 @@
     <t>PLASTIC CONTAINER 2500 ML</t>
   </si>
   <si>
-    <t>PLASTIC CONTAINER 300 ML SQURE</t>
-  </si>
-  <si>
     <t>CRATE</t>
   </si>
   <si>
-    <t>SHAWARMA BOX</t>
-  </si>
-  <si>
     <t>LAUNDRY BAG</t>
   </si>
   <si>
@@ -354,7 +291,106 @@
     <t>PH:9072112316</t>
   </si>
   <si>
-    <t>.</t>
+    <t>BIO PAPER CUP 150 ML</t>
+  </si>
+  <si>
+    <t>BIO PAPER CUP 210 ML</t>
+  </si>
+  <si>
+    <t>BIO PAPER PLATE SMALL</t>
+  </si>
+  <si>
+    <t>WOODEN SPOON 140 MM</t>
+  </si>
+  <si>
+    <t>WOODEN STIRER 140 MM</t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 300 ML</t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 500 ML ROUND</t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 1000 ML ROUND</t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 1000 ML SQUARE</t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 750 ML ROUND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOS </t>
+  </si>
+  <si>
+    <t>PLASTIC CONTAINER 500 GM/ 450 ML ROUND</t>
+  </si>
+  <si>
+    <t>JUMBO KITCHEN PAPER ROLL</t>
+  </si>
+  <si>
+    <t>BUCKET 40 LTR</t>
+  </si>
+  <si>
+    <t>TABLE CLEANING SPONGE (CELLULOSE WIPE)</t>
+  </si>
+  <si>
+    <t>WIPER (BLACK)</t>
+  </si>
+  <si>
+    <t>WIPER MULTI-COLOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLASTIC BROOM </t>
+  </si>
+  <si>
+    <t xml:space="preserve">COCONUT BROOM </t>
+  </si>
+  <si>
+    <t>MOP</t>
+  </si>
+  <si>
+    <t>SILVER POUCH</t>
+  </si>
+  <si>
+    <t>RIPPLE CUP 150 ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RIPPLE CUP 210 ML </t>
+  </si>
+  <si>
+    <t>DINE EARTH PAPER PLATE 6 INCH</t>
+  </si>
+  <si>
+    <t>PIN 25 MM</t>
+  </si>
+  <si>
+    <t>PAPER BAG (11*11*6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAPER COVER V BOTTOM </t>
+  </si>
+  <si>
+    <t>SOS PAPER COVER SQUARE BOTTOM  ( S,M,L)</t>
+  </si>
+  <si>
+    <t>5 COMPARTMENT PARCEL TRAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 COMPARTMENT PARCEL TRAY </t>
+  </si>
+  <si>
+    <t>3 COMPARTMENT PARCEL TRAY</t>
+  </si>
+  <si>
+    <t>BL PLASTIC GLASS 300 ML</t>
+  </si>
+  <si>
+    <t>BL PLASTIC GLASS 350 ML</t>
+  </si>
+  <si>
+    <t>WRAPPED STRAW 8MM</t>
   </si>
 </sst>
 </file>
@@ -542,7 +578,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -606,6 +642,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -921,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D797BD9-D84B-4EEF-82AC-4552D00F2819}">
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D116"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="2" customWidth="1"/>
@@ -931,7 +969,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="7" customFormat="1" ht="33.6" x14ac:dyDescent="0.65">
       <c r="A1" s="10" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -939,7 +977,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -947,7 +985,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
@@ -955,7 +993,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="23"/>
@@ -963,7 +1001,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="20"/>
@@ -988,7 +1026,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1002,7 +1040,7 @@
         <v>5</v>
       </c>
       <c r="D8" s="3">
-        <v>260</v>
+        <v>325</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1024,7 +1062,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>7</v>
@@ -1041,10 +1079,10 @@
         <v>9</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3">
-        <v>16</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1058,7 +1096,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="3">
-        <v>90</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1072,7 +1110,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="3">
-        <v>300</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1086,7 +1124,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="3">
-        <v>400</v>
+        <v>490</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1139,7 +1177,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" s="3">
         <v>135</v>
@@ -1150,13 +1188,13 @@
         <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1164,399 +1202,395 @@
         <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="3">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
-        <v>14</v>
-      </c>
+      <c r="A21" s="3"/>
       <c r="B21" s="1" t="s">
-        <v>17</v>
+        <v>121</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="3">
-        <v>300</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
-        <v>15</v>
-      </c>
+      <c r="A22" s="3"/>
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D22" s="3">
-        <v>280</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="3">
-        <v>25</v>
+        <v>325</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="3">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D25" s="3">
-        <v>125</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="3">
-        <v>200</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D27" s="3">
-        <v>125</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D28" s="3">
-        <v>65</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
+        <v>21</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="C29" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D29" s="3">
-        <v>180</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
+        <v>22</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="3">
-        <v>140</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
+        <v>23</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="C31" s="3" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="D31" s="3">
-        <v>330</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="D32" s="3">
-        <v>230</v>
+        <v>345</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="D33" s="3">
-        <v>195</v>
+        <v>295</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>7</v>
+        <v>68</v>
       </c>
       <c r="D34" s="3">
-        <v>380</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D35" s="3">
-        <v>14.75</v>
+        <v>390</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D36" s="3">
-        <v>105</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D37" s="3">
-        <v>30</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D38" s="3">
-        <v>12</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D39" s="3">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D40" s="3">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D41" s="3">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D42" s="3">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D43" s="3">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="D44" s="3">
-        <v>45</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D45" s="3">
-        <v>145</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D46" s="3">
-        <v>48</v>
+        <v>165</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D47" s="3">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>8</v>
@@ -1567,754 +1601,910 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>37</v>
+        <v>92</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D49" s="3">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D50" s="3">
-        <v>75</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D51" s="3">
-        <v>0.68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D52" s="3">
-        <v>1.35</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D53" s="3">
-        <v>2.15</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D54" s="3">
-        <v>3.25</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D55" s="3">
-        <v>6.5</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D56" s="3">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="D56" s="3"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D57" s="3">
-        <v>4.32</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D58" s="3">
-        <v>6.9</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D59" s="3">
-        <v>5.75</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D60" s="3">
-        <v>6</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D61" s="3">
-        <v>18.36</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D62" s="3">
-        <v>2.65</v>
+        <v>18.36</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D63" s="3">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A64" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B64" s="17"/>
-      <c r="C64" s="17"/>
-      <c r="D64" s="18"/>
+        <v>98</v>
+      </c>
+      <c r="D63" s="3"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="3"/>
+      <c r="B64" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" s="3">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="3">
-        <v>1</v>
-      </c>
+      <c r="A65" s="3"/>
       <c r="B65" s="1" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D65" s="3">
-        <v>180</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="3">
-        <v>2</v>
-      </c>
+      <c r="A66" s="3"/>
       <c r="B66" s="1" t="s">
-        <v>43</v>
+        <v>112</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D66" s="3">
-        <v>454</v>
+        <v>40</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="3">
-        <v>3</v>
-      </c>
+      <c r="A67" s="3"/>
       <c r="B67" s="1" t="s">
-        <v>44</v>
+        <v>114</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D67" s="3">
-        <v>320</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="3">
-        <v>4</v>
-      </c>
+      <c r="A68" s="3"/>
       <c r="B68" s="1" t="s">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D68" s="3">
-        <v>460</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="3">
-        <v>5</v>
-      </c>
+      <c r="A69" s="3"/>
       <c r="B69" s="1" t="s">
-        <v>46</v>
+        <v>118</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D69" s="3">
-        <v>360</v>
+        <v>12</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="3">
+      <c r="A70" s="3"/>
+      <c r="B70" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D70" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="3"/>
+      <c r="B71" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" s="3"/>
+      <c r="B72" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D72" s="3">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="3"/>
+      <c r="B73" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" s="3">
         <v>6</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D70" s="3">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="3">
-        <v>7</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D71" s="3">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="3">
-        <v>8</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D72" s="3">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="3">
-        <v>9</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D73" s="3">
-        <v>625</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="3">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D74" s="3">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="3">
-        <v>11</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D75" s="3">
-        <v>250</v>
-      </c>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="A75" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B75" s="17"/>
+      <c r="C75" s="17"/>
+      <c r="D75" s="18"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D76" s="3">
-        <v>95</v>
+        <v>290</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="3">
-        <v>13</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D77" s="3">
-        <v>65</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B77" s="1"/>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>88</v>
+        <v>34</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D78" s="3">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A79" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="15"/>
+        <v>390</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="3">
+        <v>4</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D79" s="3">
+        <v>485</v>
+      </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>106</v>
+        <v>5</v>
+      </c>
+      <c r="D80" s="3">
+        <v>445</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D81" s="3">
-        <v>42</v>
+        <v>350</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="3">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D82" s="3">
-        <v>25</v>
+        <v>649</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D83" s="3">
-        <v>37</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D84" s="3">
-        <v>48</v>
+        <v>895</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D85" s="3">
-        <v>260</v>
+        <v>230</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D86" s="3">
-        <v>220</v>
+        <v>289</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D87" s="3">
-        <v>385</v>
+        <v>110</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="3">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D88" s="3">
-        <v>115</v>
+        <v>65</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="3">
-        <v>10</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D89" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="3">
-        <v>11</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D90" s="3">
-        <v>35</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B89" s="1"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+    </row>
+    <row r="90" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+      <c r="A90" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B90" s="14"/>
+      <c r="C90" s="14"/>
+      <c r="D90" s="15"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D91" s="3">
-        <v>55</v>
+        <v>8</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="3">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D92" s="3">
-        <v>160</v>
+        <v>48</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D93" s="3">
-        <v>850</v>
+        <v>18</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="3">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D94" s="3">
-        <v>195</v>
+        <v>37</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="3">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D95" s="3">
-        <v>220</v>
+        <v>315</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="3">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D96" s="3">
-        <v>35</v>
+        <v>300</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>65</v>
+        <v>103</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D97" s="3">
-        <v>560</v>
+        <v>260</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="3">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D98" s="3">
-        <v>36</v>
+        <v>325</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="3">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D99" s="3">
-        <v>185</v>
+        <v>120</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="3">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D100" s="3">
-        <v>11.25</v>
+        <v>99</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="3">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>103</v>
+        <v>46</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D101" s="3">
-        <v>32</v>
+        <v>65</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="3">
+        <v>12</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D102" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" s="3">
+        <v>13</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D103" s="3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" s="3">
+        <v>14</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D104" s="3">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A105" s="3">
+        <v>15</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D105" s="3">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A106" s="3">
+        <v>16</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D106" s="3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A107" s="3">
+        <v>17</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D107" s="3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A108" s="3">
+        <v>18</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D108" s="3">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A109" s="3">
+        <v>19</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D109" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A110" s="3">
+        <v>20</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D110" s="3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A111" s="3">
+        <v>21</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D111" s="3">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A112" s="3">
+        <v>22</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D112" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" s="3">
         <v>23</v>
       </c>
-      <c r="B102" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D102" s="3">
+      <c r="B113" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D113" s="3">
         <v>315</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A114" s="2">
+        <v>24</v>
+      </c>
+      <c r="B114" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D114" s="2">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A115" s="2">
+        <v>25</v>
+      </c>
+      <c r="B115" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D115" s="2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" s="2">
+        <v>26</v>
+      </c>
+      <c r="B116" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D116" s="2">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A75:D75"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A79:D79"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:D4"/>

</xml_diff>